<commit_message>
chore(auto): daily B2B surplus feeds, REST API, compliance & SEO refresh
</commit_message>
<xml_diff>
--- a/exports/Florida_Surplus_Feed.xlsx
+++ b/exports/Florida_Surplus_Feed.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N13"/>
+  <dimension ref="A1:Q13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -454,35 +454,50 @@
       </c>
       <c r="H1" t="inlineStr">
         <is>
+          <t>Property_Type</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
           <t>Surplus_Balance_USD</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Statutory_Fee_Rate</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Est_Finder_Fee_USD</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Opportunity_Tier</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Sale_Date</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
+        <is>
+          <t>Statutory_Deadline_Window</t>
+        </is>
+      </c>
+      <c r="O1" t="inlineStr">
+        <is>
+          <t>Clerk_Verification_URL</t>
+        </is>
+      </c>
+      <c r="P1" t="inlineStr">
         <is>
           <t>Governing_Statute</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Enriched_Timestamp</t>
         </is>
@@ -522,35 +537,50 @@
           <t>720 S OCEAN BLVD PALM BEACH FL 33480</t>
         </is>
       </c>
-      <c r="H2" t="n">
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>Commercial / Mixed Use</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
         <v>145000</v>
       </c>
-      <c r="I2" t="inlineStr">
+      <c r="J2" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J2" t="n">
+      <c r="K2" t="n">
         <v>29000</v>
       </c>
-      <c r="K2" t="inlineStr">
+      <c r="L2" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>2024-06-28</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>https://www.mypalmbeachclerk.com/</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -588,35 +618,50 @@
           <t>340 SW 8TH ST MIAMI FL 33130</t>
         </is>
       </c>
-      <c r="H3" t="n">
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
         <v>112000</v>
       </c>
-      <c r="I3" t="inlineStr">
+      <c r="J3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J3" t="n">
+      <c r="K3" t="n">
         <v>22400</v>
       </c>
-      <c r="K3" t="inlineStr">
+      <c r="L3" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>2024-08-05</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>https://www.miamidadeclerk.gov/</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -654,35 +699,50 @@
           <t>4502 W SAN RAFAEL ST TAMPA FL 33629</t>
         </is>
       </c>
-      <c r="H4" t="n">
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
         <v>92400</v>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="J4" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J4" t="n">
+      <c r="K4" t="n">
         <v>18480</v>
       </c>
-      <c r="K4" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>2024-07-25</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O4" t="inlineStr">
+        <is>
+          <t>https://www.hillsclerk.com/</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q4" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -720,35 +780,50 @@
           <t>8431 BAY BREEZE WAY ORLANDO FL 32836</t>
         </is>
       </c>
-      <c r="H5" t="n">
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>74300</v>
       </c>
-      <c r="I5" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J5" t="n">
+      <c r="K5" t="n">
         <v>14860</v>
       </c>
-      <c r="K5" t="inlineStr">
+      <c r="L5" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>2024-08-08</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>https://www.myorangeclerk.com/</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q5" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -786,35 +861,50 @@
           <t>1410 N FEDERAL HWY LAKE WORTH FL 33460</t>
         </is>
       </c>
-      <c r="H6" t="n">
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>Commercial / Mixed Use</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>68900</v>
       </c>
-      <c r="I6" t="inlineStr">
+      <c r="J6" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J6" t="n">
+      <c r="K6" t="n">
         <v>13780</v>
       </c>
-      <c r="K6" t="inlineStr">
+      <c r="L6" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>2024-07-14</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O6" t="inlineStr">
+        <is>
+          <t>https://www.mypalmbeachclerk.com/</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q6" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -852,35 +942,50 @@
           <t>3309 ROSEWOOD CT WINTER PARK FL 32792</t>
         </is>
       </c>
-      <c r="H7" t="n">
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>61800</v>
       </c>
-      <c r="I7" t="inlineStr">
+      <c r="J7" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J7" t="n">
+      <c r="K7" t="n">
         <v>12360</v>
       </c>
-      <c r="K7" t="inlineStr">
+      <c r="L7" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>2024-07-03</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>https://www.myorangeclerk.com/</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -918,35 +1023,50 @@
           <t>11804 N 56TH ST TEMPLE TERRACE FL 33617</t>
         </is>
       </c>
-      <c r="H8" t="n">
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>54100</v>
       </c>
-      <c r="I8" t="inlineStr">
+      <c r="J8" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J8" t="n">
+      <c r="K8" t="n">
         <v>10820</v>
       </c>
-      <c r="K8" t="inlineStr">
+      <c r="L8" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>2024-08-02</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>https://www.hillsclerk.com/</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -984,35 +1104,50 @@
           <t>1420 PINEWOOD DR ORLANDO FL 32808</t>
         </is>
       </c>
-      <c r="H9" t="n">
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>48250</v>
       </c>
-      <c r="I9" t="inlineStr">
+      <c r="J9" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J9" t="n">
+      <c r="K9" t="n">
         <v>9650</v>
       </c>
-      <c r="K9" t="inlineStr">
+      <c r="L9" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>2024-06-12</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>https://www.myorangeclerk.com/</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -1050,35 +1185,50 @@
           <t>1920 CORAL WAY MIAMI FL 33145</t>
         </is>
       </c>
-      <c r="H10" t="n">
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>43500</v>
       </c>
-      <c r="I10" t="inlineStr">
+      <c r="J10" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J10" t="n">
+      <c r="K10" t="n">
         <v>8700</v>
       </c>
-      <c r="K10" t="inlineStr">
+      <c r="L10" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>2024-08-12</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>https://www.miamidadeclerk.gov/</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -1116,35 +1266,50 @@
           <t>2308 S ARMENIA AVE TAMPA FL 33629</t>
         </is>
       </c>
-      <c r="H11" t="n">
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>31750</v>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="J11" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J11" t="n">
+      <c r="K11" t="n">
         <v>6350</v>
       </c>
-      <c r="K11" t="inlineStr">
+      <c r="L11" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>2024-08-10</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>https://www.hillsclerk.com/</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -1182,35 +1347,50 @@
           <t>510 LAKE BREEZE DR APOPKA FL 32703</t>
         </is>
       </c>
-      <c r="H12" t="n">
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>29400</v>
       </c>
-      <c r="I12" t="inlineStr">
+      <c r="J12" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J12" t="n">
+      <c r="K12" t="n">
         <v>5880</v>
       </c>
-      <c r="K12" t="inlineStr">
+      <c r="L12" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>2024-07-17</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>https://www.myorangeclerk.com/</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>
@@ -1248,35 +1428,50 @@
           <t>220 W KALEY ST ORLANDO FL 32806</t>
         </is>
       </c>
-      <c r="H13" t="n">
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>Single Family Residential</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>18900</v>
       </c>
-      <c r="I13" t="inlineStr">
+      <c r="J13" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="J13" t="n">
+      <c r="K13" t="n">
         <v>3780</v>
       </c>
-      <c r="K13" t="inlineStr">
+      <c r="L13" t="inlineStr">
         <is>
           <t>Tier 2: Medium Value ($10k-$25k)</t>
         </is>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>2024-08-01</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>120 Days from Notice (FL Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>https://www.myorangeclerk.com/</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
         <is>
           <t>FL Statute § 197.582</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>2026-08-22 11:12:30</t>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>2026-08-23 12:56:15</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(audit): resolve county breadcrumb links, add canonical utility tags, and update state Excel feeds
</commit_message>
<xml_diff>
--- a/exports/Florida_Surplus_Feed.xlsx
+++ b/exports/Florida_Surplus_Feed.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Q13"/>
+  <dimension ref="A1:R13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -449,55 +449,60 @@
       </c>
       <c r="G1" t="inlineStr">
         <is>
+          <t>Heir_Search_Recommended</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
           <t>Property_Address</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>Property_Type</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>Surplus_Balance_USD</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>Statutory_Fee_Rate</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>Est_Finder_Fee_USD</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>Opportunity_Tier</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>Sale_Date</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>Statutory_Deadline_Window</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>Clerk_Verification_URL</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>Governing_Statute</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>Enriched_Timestamp</t>
         </is>
@@ -532,55 +537,58 @@
       <c r="F2" t="b">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" t="b">
+        <v>0</v>
+      </c>
+      <c r="H2" t="inlineStr">
         <is>
           <t>720 S OCEAN BLVD PALM BEACH FL 33480</t>
         </is>
       </c>
-      <c r="H2" t="inlineStr">
+      <c r="I2" t="inlineStr">
         <is>
           <t>Commercial / Mixed Use</t>
         </is>
       </c>
-      <c r="I2" t="n">
+      <c r="J2" t="n">
         <v>145000</v>
       </c>
-      <c r="J2" t="inlineStr">
+      <c r="K2" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K2" t="n">
+      <c r="L2" t="n">
         <v>29000</v>
       </c>
-      <c r="L2" t="inlineStr">
+      <c r="M2" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M2" t="inlineStr">
+      <c r="N2" t="inlineStr">
         <is>
           <t>2024-06-28</t>
         </is>
       </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O2" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
           <t>https://www.mypalmbeachclerk.com/</t>
         </is>
       </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q2" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -613,55 +621,58 @@
       <c r="F3" t="b">
         <v>1</v>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="G3" t="b">
+        <v>0</v>
+      </c>
+      <c r="H3" t="inlineStr">
         <is>
           <t>340 SW 8TH ST MIAMI FL 33130</t>
         </is>
       </c>
-      <c r="H3" t="inlineStr">
+      <c r="I3" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I3" t="n">
+      <c r="J3" t="n">
         <v>112000</v>
       </c>
-      <c r="J3" t="inlineStr">
+      <c r="K3" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K3" t="n">
+      <c r="L3" t="n">
         <v>22400</v>
       </c>
-      <c r="L3" t="inlineStr">
+      <c r="M3" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M3" t="inlineStr">
+      <c r="N3" t="inlineStr">
         <is>
           <t>2024-08-05</t>
         </is>
       </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O3" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
           <t>https://www.miamidadeclerk.gov/</t>
         </is>
       </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q3" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -694,55 +705,58 @@
       <c r="F4" t="b">
         <v>1</v>
       </c>
-      <c r="G4" t="inlineStr">
+      <c r="G4" t="b">
+        <v>0</v>
+      </c>
+      <c r="H4" t="inlineStr">
         <is>
           <t>4502 W SAN RAFAEL ST TAMPA FL 33629</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr">
+      <c r="I4" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I4" t="n">
+      <c r="J4" t="n">
         <v>92400</v>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="K4" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K4" t="n">
+      <c r="L4" t="n">
         <v>18480</v>
       </c>
-      <c r="L4" t="inlineStr">
+      <c r="M4" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M4" t="inlineStr">
+      <c r="N4" t="inlineStr">
         <is>
           <t>2024-07-25</t>
         </is>
       </c>
-      <c r="N4" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O4" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P4" t="inlineStr">
+        <is>
           <t>https://www.hillsclerk.com/</t>
         </is>
       </c>
-      <c r="P4" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q4" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R4" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -775,55 +789,58 @@
       <c r="F5" t="b">
         <v>1</v>
       </c>
-      <c r="G5" t="inlineStr">
+      <c r="G5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>8431 BAY BREEZE WAY ORLANDO FL 32836</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I5" t="n">
+      <c r="J5" t="n">
         <v>74300</v>
       </c>
-      <c r="J5" t="inlineStr">
+      <c r="K5" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K5" t="n">
+      <c r="L5" t="n">
         <v>14860</v>
       </c>
-      <c r="L5" t="inlineStr">
+      <c r="M5" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M5" t="inlineStr">
+      <c r="N5" t="inlineStr">
         <is>
           <t>2024-08-08</t>
         </is>
       </c>
-      <c r="N5" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O5" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P5" t="inlineStr">
+        <is>
           <t>https://www.myorangeclerk.com/</t>
         </is>
       </c>
-      <c r="P5" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q5" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R5" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -856,55 +873,58 @@
       <c r="F6" t="b">
         <v>1</v>
       </c>
-      <c r="G6" t="inlineStr">
+      <c r="G6" t="b">
+        <v>1</v>
+      </c>
+      <c r="H6" t="inlineStr">
         <is>
           <t>1410 N FEDERAL HWY LAKE WORTH FL 33460</t>
         </is>
       </c>
-      <c r="H6" t="inlineStr">
+      <c r="I6" t="inlineStr">
         <is>
           <t>Commercial / Mixed Use</t>
         </is>
       </c>
-      <c r="I6" t="n">
+      <c r="J6" t="n">
         <v>68900</v>
       </c>
-      <c r="J6" t="inlineStr">
+      <c r="K6" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K6" t="n">
+      <c r="L6" t="n">
         <v>13780</v>
       </c>
-      <c r="L6" t="inlineStr">
+      <c r="M6" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M6" t="inlineStr">
+      <c r="N6" t="inlineStr">
         <is>
           <t>2024-07-14</t>
         </is>
       </c>
-      <c r="N6" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O6" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P6" t="inlineStr">
+        <is>
           <t>https://www.mypalmbeachclerk.com/</t>
         </is>
       </c>
-      <c r="P6" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q6" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R6" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -937,55 +957,58 @@
       <c r="F7" t="b">
         <v>1</v>
       </c>
-      <c r="G7" t="inlineStr">
+      <c r="G7" t="b">
+        <v>1</v>
+      </c>
+      <c r="H7" t="inlineStr">
         <is>
           <t>3309 ROSEWOOD CT WINTER PARK FL 32792</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr">
+      <c r="I7" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I7" t="n">
+      <c r="J7" t="n">
         <v>61800</v>
       </c>
-      <c r="J7" t="inlineStr">
+      <c r="K7" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K7" t="n">
+      <c r="L7" t="n">
         <v>12360</v>
       </c>
-      <c r="L7" t="inlineStr">
+      <c r="M7" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M7" t="inlineStr">
+      <c r="N7" t="inlineStr">
         <is>
           <t>2024-07-03</t>
         </is>
       </c>
-      <c r="N7" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O7" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
           <t>https://www.myorangeclerk.com/</t>
         </is>
       </c>
-      <c r="P7" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q7" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -1018,55 +1041,58 @@
       <c r="F8" t="b">
         <v>1</v>
       </c>
-      <c r="G8" t="inlineStr">
+      <c r="G8" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" t="inlineStr">
         <is>
           <t>11804 N 56TH ST TEMPLE TERRACE FL 33617</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr">
+      <c r="I8" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I8" t="n">
+      <c r="J8" t="n">
         <v>54100</v>
       </c>
-      <c r="J8" t="inlineStr">
+      <c r="K8" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K8" t="n">
+      <c r="L8" t="n">
         <v>10820</v>
       </c>
-      <c r="L8" t="inlineStr">
+      <c r="M8" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M8" t="inlineStr">
+      <c r="N8" t="inlineStr">
         <is>
           <t>2024-08-02</t>
         </is>
       </c>
-      <c r="N8" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O8" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
           <t>https://www.hillsclerk.com/</t>
         </is>
       </c>
-      <c r="P8" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q8" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -1099,55 +1125,58 @@
       <c r="F9" t="b">
         <v>1</v>
       </c>
-      <c r="G9" t="inlineStr">
+      <c r="G9" t="b">
+        <v>0</v>
+      </c>
+      <c r="H9" t="inlineStr">
         <is>
           <t>1420 PINEWOOD DR ORLANDO FL 32808</t>
         </is>
       </c>
-      <c r="H9" t="inlineStr">
+      <c r="I9" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I9" t="n">
+      <c r="J9" t="n">
         <v>48250</v>
       </c>
-      <c r="J9" t="inlineStr">
+      <c r="K9" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K9" t="n">
+      <c r="L9" t="n">
         <v>9650</v>
       </c>
-      <c r="L9" t="inlineStr">
+      <c r="M9" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M9" t="inlineStr">
+      <c r="N9" t="inlineStr">
         <is>
           <t>2024-06-12</t>
         </is>
       </c>
-      <c r="N9" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O9" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
           <t>https://www.myorangeclerk.com/</t>
         </is>
       </c>
-      <c r="P9" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q9" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -1180,55 +1209,58 @@
       <c r="F10" t="b">
         <v>1</v>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G10" t="b">
+        <v>0</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>1920 CORAL WAY MIAMI FL 33145</t>
         </is>
       </c>
-      <c r="H10" t="inlineStr">
+      <c r="I10" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I10" t="n">
+      <c r="J10" t="n">
         <v>43500</v>
       </c>
-      <c r="J10" t="inlineStr">
+      <c r="K10" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K10" t="n">
+      <c r="L10" t="n">
         <v>8700</v>
       </c>
-      <c r="L10" t="inlineStr">
+      <c r="M10" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M10" t="inlineStr">
+      <c r="N10" t="inlineStr">
         <is>
           <t>2024-08-12</t>
         </is>
       </c>
-      <c r="N10" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O10" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
           <t>https://www.miamidadeclerk.gov/</t>
         </is>
       </c>
-      <c r="P10" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q10" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -1261,55 +1293,58 @@
       <c r="F11" t="b">
         <v>1</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G11" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>2308 S ARMENIA AVE TAMPA FL 33629</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="I11" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I11" t="n">
+      <c r="J11" t="n">
         <v>31750</v>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="K11" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K11" t="n">
+      <c r="L11" t="n">
         <v>6350</v>
       </c>
-      <c r="L11" t="inlineStr">
+      <c r="M11" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M11" t="inlineStr">
+      <c r="N11" t="inlineStr">
         <is>
           <t>2024-08-10</t>
         </is>
       </c>
-      <c r="N11" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O11" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
           <t>https://www.hillsclerk.com/</t>
         </is>
       </c>
-      <c r="P11" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q11" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -1342,55 +1377,58 @@
       <c r="F12" t="b">
         <v>1</v>
       </c>
-      <c r="G12" t="inlineStr">
+      <c r="G12" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" t="inlineStr">
         <is>
           <t>510 LAKE BREEZE DR APOPKA FL 32703</t>
         </is>
       </c>
-      <c r="H12" t="inlineStr">
+      <c r="I12" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I12" t="n">
+      <c r="J12" t="n">
         <v>29400</v>
       </c>
-      <c r="J12" t="inlineStr">
+      <c r="K12" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K12" t="n">
+      <c r="L12" t="n">
         <v>5880</v>
       </c>
-      <c r="L12" t="inlineStr">
+      <c r="M12" t="inlineStr">
         <is>
           <t>Tier 1: High Value ($25k+)</t>
         </is>
       </c>
-      <c r="M12" t="inlineStr">
+      <c r="N12" t="inlineStr">
         <is>
           <t>2024-07-17</t>
         </is>
       </c>
-      <c r="N12" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O12" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
           <t>https://www.myorangeclerk.com/</t>
         </is>
       </c>
-      <c r="P12" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q12" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>
@@ -1423,55 +1461,58 @@
       <c r="F13" t="b">
         <v>1</v>
       </c>
-      <c r="G13" t="inlineStr">
+      <c r="G13" t="b">
+        <v>0</v>
+      </c>
+      <c r="H13" t="inlineStr">
         <is>
           <t>220 W KALEY ST ORLANDO FL 32806</t>
         </is>
       </c>
-      <c r="H13" t="inlineStr">
+      <c r="I13" t="inlineStr">
         <is>
           <t>Single Family Residential</t>
         </is>
       </c>
-      <c r="I13" t="n">
+      <c r="J13" t="n">
         <v>18900</v>
       </c>
-      <c r="J13" t="inlineStr">
+      <c r="K13" t="inlineStr">
         <is>
           <t>20%</t>
         </is>
       </c>
-      <c r="K13" t="n">
+      <c r="L13" t="n">
         <v>3780</v>
       </c>
-      <c r="L13" t="inlineStr">
+      <c r="M13" t="inlineStr">
         <is>
           <t>Tier 2: Medium Value ($10k-$25k)</t>
         </is>
       </c>
-      <c r="M13" t="inlineStr">
+      <c r="N13" t="inlineStr">
         <is>
           <t>2024-08-01</t>
         </is>
       </c>
-      <c r="N13" t="inlineStr">
-        <is>
-          <t>120 Days from Notice (FL Stat. § 197.582)</t>
-        </is>
-      </c>
       <c r="O13" t="inlineStr">
         <is>
+          <t>120 Days from Notice (Fla. Stat. § 197.582)</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
           <t>https://www.myorangeclerk.com/</t>
         </is>
       </c>
-      <c r="P13" t="inlineStr">
-        <is>
-          <t>FL Statute § 197.582</t>
-        </is>
-      </c>
       <c r="Q13" t="inlineStr">
         <is>
-          <t>2026-08-25 11:18:14</t>
+          <t>Fla. Stat. § 197.582</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>2026-08-25 10:41:32</t>
         </is>
       </c>
     </row>

</xml_diff>